<commit_message>
chore: workbook Status = Ready, Verified = Yes for all 33 assets
Every workbook asset is delivered and imports correctly in the 3D frontend
(all 42 manifest entries and the skybox load on /assets, 2026-10-05).
Only the Status (E2:E34) and Verified (I2:I34) cells changed; ownership,
priority and every other cell and zip entry are byte-identical.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/3d_models/EmergencyFlow_3D_Asset_Checklist_Assigned.xlsx
+++ b/3d_models/EmergencyFlow_3D_Asset_Checklist_Assigned.xlsx
@@ -741,7 +741,7 @@
       </x:c>
       <x:c r="E2" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
+          <x:t xml:space="preserve">Ready</x:t>
         </x:is>
       </x:c>
       <x:c r="F2" s="2" t="str">
@@ -759,7 +759,7 @@
       </x:c>
       <x:c r="I2" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">No</x:t>
+          <x:t xml:space="preserve">Yes</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -786,7 +786,7 @@
       </x:c>
       <x:c r="E3" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
+          <x:t xml:space="preserve">Ready</x:t>
         </x:is>
       </x:c>
       <x:c r="F3" s="2" t="str">
@@ -804,7 +804,7 @@
       </x:c>
       <x:c r="I3" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">No</x:t>
+          <x:t xml:space="preserve">Yes</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -831,7 +831,7 @@
       </x:c>
       <x:c r="E4" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
+          <x:t xml:space="preserve">Ready</x:t>
         </x:is>
       </x:c>
       <x:c r="F4" s="2" t="str">
@@ -849,7 +849,7 @@
       </x:c>
       <x:c r="I4" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">No</x:t>
+          <x:t xml:space="preserve">Yes</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -876,7 +876,7 @@
       </x:c>
       <x:c r="E5" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
+          <x:t xml:space="preserve">Ready</x:t>
         </x:is>
       </x:c>
       <x:c r="F5" s="2" t="str">
@@ -894,7 +894,7 @@
       </x:c>
       <x:c r="I5" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">No</x:t>
+          <x:t xml:space="preserve">Yes</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -921,7 +921,7 @@
       </x:c>
       <x:c r="E6" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
+          <x:t xml:space="preserve">Ready</x:t>
         </x:is>
       </x:c>
       <x:c r="F6" s="2" t="str">
@@ -939,7 +939,7 @@
       </x:c>
       <x:c r="I6" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">No</x:t>
+          <x:t xml:space="preserve">Yes</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -966,7 +966,7 @@
       </x:c>
       <x:c r="E7" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
+          <x:t xml:space="preserve">Ready</x:t>
         </x:is>
       </x:c>
       <x:c r="F7" s="2" t="str">
@@ -984,7 +984,7 @@
       </x:c>
       <x:c r="I7" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">No</x:t>
+          <x:t xml:space="preserve">Yes</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1011,7 +1011,7 @@
       </x:c>
       <x:c r="E8" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
+          <x:t xml:space="preserve">Ready</x:t>
         </x:is>
       </x:c>
       <x:c r="F8" s="2" t="str">
@@ -1029,7 +1029,7 @@
       </x:c>
       <x:c r="I8" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">No</x:t>
+          <x:t xml:space="preserve">Yes</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1056,7 +1056,7 @@
       </x:c>
       <x:c r="E9" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
+          <x:t xml:space="preserve">Ready</x:t>
         </x:is>
       </x:c>
       <x:c r="F9" s="2" t="str">
@@ -1074,7 +1074,7 @@
       </x:c>
       <x:c r="I9" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">No</x:t>
+          <x:t xml:space="preserve">Yes</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1101,7 +1101,7 @@
       </x:c>
       <x:c r="E10" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
+          <x:t xml:space="preserve">Ready</x:t>
         </x:is>
       </x:c>
       <x:c r="F10" s="2" t="str">
@@ -1119,7 +1119,7 @@
       </x:c>
       <x:c r="I10" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">No</x:t>
+          <x:t xml:space="preserve">Yes</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1146,7 +1146,7 @@
       </x:c>
       <x:c r="E11" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
+          <x:t xml:space="preserve">Ready</x:t>
         </x:is>
       </x:c>
       <x:c r="F11" s="2" t="str">
@@ -1164,7 +1164,7 @@
       </x:c>
       <x:c r="I11" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">No</x:t>
+          <x:t xml:space="preserve">Yes</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1191,7 +1191,7 @@
       </x:c>
       <x:c r="E12" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
+          <x:t xml:space="preserve">Ready</x:t>
         </x:is>
       </x:c>
       <x:c r="F12" s="2" t="str">
@@ -1209,7 +1209,7 @@
       </x:c>
       <x:c r="I12" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">No</x:t>
+          <x:t xml:space="preserve">Yes</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1236,7 +1236,7 @@
       </x:c>
       <x:c r="E13" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
+          <x:t xml:space="preserve">Ready</x:t>
         </x:is>
       </x:c>
       <x:c r="F13" s="2" t="str">
@@ -1254,7 +1254,7 @@
       </x:c>
       <x:c r="I13" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">No</x:t>
+          <x:t xml:space="preserve">Yes</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1281,7 +1281,7 @@
       </x:c>
       <x:c r="E14" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
+          <x:t xml:space="preserve">Ready</x:t>
         </x:is>
       </x:c>
       <x:c r="F14" s="2" t="str">
@@ -1299,7 +1299,7 @@
       </x:c>
       <x:c r="I14" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">No</x:t>
+          <x:t xml:space="preserve">Yes</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1326,7 +1326,7 @@
       </x:c>
       <x:c r="E15" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
+          <x:t xml:space="preserve">Ready</x:t>
         </x:is>
       </x:c>
       <x:c r="F15" s="2" t="str">
@@ -1344,7 +1344,7 @@
       </x:c>
       <x:c r="I15" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">No</x:t>
+          <x:t xml:space="preserve">Yes</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1371,7 +1371,7 @@
       </x:c>
       <x:c r="E16" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
+          <x:t xml:space="preserve">Ready</x:t>
         </x:is>
       </x:c>
       <x:c r="F16" s="2" t="str">
@@ -1389,7 +1389,7 @@
       </x:c>
       <x:c r="I16" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">No</x:t>
+          <x:t xml:space="preserve">Yes</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1416,7 +1416,7 @@
       </x:c>
       <x:c r="E17" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
+          <x:t xml:space="preserve">Ready</x:t>
         </x:is>
       </x:c>
       <x:c r="F17" s="2" t="str">
@@ -1434,7 +1434,7 @@
       </x:c>
       <x:c r="I17" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">No</x:t>
+          <x:t xml:space="preserve">Yes</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1461,7 +1461,7 @@
       </x:c>
       <x:c r="E18" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
+          <x:t xml:space="preserve">Ready</x:t>
         </x:is>
       </x:c>
       <x:c r="F18" s="2" t="str">
@@ -1479,7 +1479,7 @@
       </x:c>
       <x:c r="I18" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">No</x:t>
+          <x:t xml:space="preserve">Yes</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1506,7 +1506,7 @@
       </x:c>
       <x:c r="E19" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
+          <x:t xml:space="preserve">Ready</x:t>
         </x:is>
       </x:c>
       <x:c r="F19" s="2" t="str">
@@ -1524,7 +1524,7 @@
       </x:c>
       <x:c r="I19" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">No</x:t>
+          <x:t xml:space="preserve">Yes</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1551,7 +1551,7 @@
       </x:c>
       <x:c r="E20" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
+          <x:t xml:space="preserve">Ready</x:t>
         </x:is>
       </x:c>
       <x:c r="F20" s="2" t="str">
@@ -1569,7 +1569,7 @@
       </x:c>
       <x:c r="I20" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">No</x:t>
+          <x:t xml:space="preserve">Yes</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1596,7 +1596,7 @@
       </x:c>
       <x:c r="E21" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
+          <x:t xml:space="preserve">Ready</x:t>
         </x:is>
       </x:c>
       <x:c r="F21" s="2" t="str">
@@ -1614,7 +1614,7 @@
       </x:c>
       <x:c r="I21" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">No</x:t>
+          <x:t xml:space="preserve">Yes</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1641,7 +1641,7 @@
       </x:c>
       <x:c r="E22" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
+          <x:t xml:space="preserve">Ready</x:t>
         </x:is>
       </x:c>
       <x:c r="F22" s="2" t="str">
@@ -1659,7 +1659,7 @@
       </x:c>
       <x:c r="I22" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">No</x:t>
+          <x:t xml:space="preserve">Yes</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1686,7 +1686,7 @@
       </x:c>
       <x:c r="E23" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
+          <x:t xml:space="preserve">Ready</x:t>
         </x:is>
       </x:c>
       <x:c r="F23" s="2" t="str">
@@ -1704,7 +1704,7 @@
       </x:c>
       <x:c r="I23" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">No</x:t>
+          <x:t xml:space="preserve">Yes</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1731,7 +1731,7 @@
       </x:c>
       <x:c r="E24" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
+          <x:t xml:space="preserve">Ready</x:t>
         </x:is>
       </x:c>
       <x:c r="F24" s="2" t="str">
@@ -1749,7 +1749,7 @@
       </x:c>
       <x:c r="I24" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">No</x:t>
+          <x:t xml:space="preserve">Yes</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1776,7 +1776,7 @@
       </x:c>
       <x:c r="E25" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
+          <x:t xml:space="preserve">Ready</x:t>
         </x:is>
       </x:c>
       <x:c r="F25" s="2" t="str">
@@ -1794,7 +1794,7 @@
       </x:c>
       <x:c r="I25" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">No</x:t>
+          <x:t xml:space="preserve">Yes</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1821,7 +1821,7 @@
       </x:c>
       <x:c r="E26" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
+          <x:t xml:space="preserve">Ready</x:t>
         </x:is>
       </x:c>
       <x:c r="F26" s="2" t="str">
@@ -1839,7 +1839,7 @@
       </x:c>
       <x:c r="I26" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">No</x:t>
+          <x:t xml:space="preserve">Yes</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1866,7 +1866,7 @@
       </x:c>
       <x:c r="E27" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
+          <x:t xml:space="preserve">Ready</x:t>
         </x:is>
       </x:c>
       <x:c r="F27" s="2" t="str">
@@ -1884,7 +1884,7 @@
       </x:c>
       <x:c r="I27" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">No</x:t>
+          <x:t xml:space="preserve">Yes</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1911,7 +1911,7 @@
       </x:c>
       <x:c r="E28" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
+          <x:t xml:space="preserve">Ready</x:t>
         </x:is>
       </x:c>
       <x:c r="F28" s="2" t="str">
@@ -1929,7 +1929,7 @@
       </x:c>
       <x:c r="I28" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">No</x:t>
+          <x:t xml:space="preserve">Yes</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1956,7 +1956,7 @@
       </x:c>
       <x:c r="E29" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
+          <x:t xml:space="preserve">Ready</x:t>
         </x:is>
       </x:c>
       <x:c r="F29" s="2" t="str">
@@ -1974,7 +1974,7 @@
       </x:c>
       <x:c r="I29" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">No</x:t>
+          <x:t xml:space="preserve">Yes</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -2001,7 +2001,7 @@
       </x:c>
       <x:c r="E30" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
+          <x:t xml:space="preserve">Ready</x:t>
         </x:is>
       </x:c>
       <x:c r="F30" s="2" t="str">
@@ -2019,7 +2019,7 @@
       </x:c>
       <x:c r="I30" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">No</x:t>
+          <x:t xml:space="preserve">Yes</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -2046,7 +2046,7 @@
       </x:c>
       <x:c r="E31" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
+          <x:t xml:space="preserve">Ready</x:t>
         </x:is>
       </x:c>
       <x:c r="F31" s="2" t="str">
@@ -2064,7 +2064,7 @@
       </x:c>
       <x:c r="I31" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">No</x:t>
+          <x:t xml:space="preserve">Yes</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -2091,7 +2091,7 @@
       </x:c>
       <x:c r="E32" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
+          <x:t xml:space="preserve">Ready</x:t>
         </x:is>
       </x:c>
       <x:c r="F32" s="2" t="str">
@@ -2109,7 +2109,7 @@
       </x:c>
       <x:c r="I32" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">No</x:t>
+          <x:t xml:space="preserve">Yes</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -2136,7 +2136,7 @@
       </x:c>
       <x:c r="E33" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
+          <x:t xml:space="preserve">Ready</x:t>
         </x:is>
       </x:c>
       <x:c r="F33" s="2" t="str">
@@ -2154,7 +2154,7 @@
       </x:c>
       <x:c r="I33" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">No</x:t>
+          <x:t xml:space="preserve">Yes</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -2181,7 +2181,7 @@
       </x:c>
       <x:c r="E34" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
+          <x:t xml:space="preserve">Ready</x:t>
         </x:is>
       </x:c>
       <x:c r="F34" s="2" t="str">
@@ -2199,7 +2199,7 @@
       </x:c>
       <x:c r="I34" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">No</x:t>
+          <x:t xml:space="preserve">Yes</x:t>
         </x:is>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
chore: workbook Team Assignments status Ready for all members; Summary counts match
The per-member Status column still said Not Started while every asset is
Ready and Verified on the main sheet. Only Team Assignments F2:F13 and the
cached results of the Summary sheet's status COUNTIFs changed.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/3d_models/EmergencyFlow_3D_Asset_Checklist_Assigned.xlsx
+++ b/3d_models/EmergencyFlow_3D_Asset_Checklist_Assigned.xlsx
@@ -2311,7 +2311,7 @@
       </x:c>
       <x:c r="B5" t="n">
         <x:f>COUNTIF('Asset Checklist'!E2:E34,"Ready")</x:f>
-        <x:v>0</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="D5" t="inlineStr">
         <x:is>
@@ -2320,7 +2320,7 @@
       </x:c>
       <x:c r="E5" t="n">
         <x:f>COUNTIF('Asset Checklist'!E2:E34,"Not Started")</x:f>
-        <x:v>33</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -2362,7 +2362,7 @@
       </x:c>
       <x:c r="E8" t="n">
         <x:f>COUNTIF('Asset Checklist'!E2:E34,"Not Started")</x:f>
-        <x:v>33</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -2402,7 +2402,7 @@
       </x:c>
       <x:c r="E10" t="n">
         <x:f>COUNTIF('Asset Checklist'!E2:E34,"Ready")</x:f>
-        <x:v>0</x:v>
+        <x:v>33</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -2545,7 +2545,7 @@
         <x:v>Core / demo-critical assets</x:v>
       </x:c>
       <x:c r="F2" s="27" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Ready</x:v>
       </x:c>
       <x:c r="G2" s="26"/>
     </x:row>
@@ -2566,7 +2566,7 @@
         <x:v>Core / demo-critical assets</x:v>
       </x:c>
       <x:c r="F3" s="27" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Ready</x:v>
       </x:c>
       <x:c r="G3" s="26"/>
     </x:row>
@@ -2587,7 +2587,7 @@
         <x:v>Core / demo-critical assets</x:v>
       </x:c>
       <x:c r="F4" s="27" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Ready</x:v>
       </x:c>
       <x:c r="G4" s="26"/>
     </x:row>
@@ -2608,7 +2608,7 @@
         <x:v>Core / demo-critical assets</x:v>
       </x:c>
       <x:c r="F5" s="27" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Ready</x:v>
       </x:c>
       <x:c r="G5" s="26"/>
     </x:row>
@@ -2629,7 +2629,7 @@
         <x:v>Traffic / incident / environment assets</x:v>
       </x:c>
       <x:c r="F6" s="27" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Ready</x:v>
       </x:c>
       <x:c r="G6" s="26"/>
     </x:row>
@@ -2650,7 +2650,7 @@
         <x:v>Traffic / incident / environment assets</x:v>
       </x:c>
       <x:c r="F7" s="27" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Ready</x:v>
       </x:c>
       <x:c r="G7" s="26"/>
     </x:row>
@@ -2671,7 +2671,7 @@
         <x:v>Traffic / incident / environment assets</x:v>
       </x:c>
       <x:c r="F8" s="27" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Ready</x:v>
       </x:c>
       <x:c r="G8" s="26"/>
     </x:row>
@@ -2692,7 +2692,7 @@
         <x:v>Traffic / incident / environment assets</x:v>
       </x:c>
       <x:c r="F9" s="27" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Ready</x:v>
       </x:c>
       <x:c r="G9" s="26"/>
     </x:row>
@@ -2713,7 +2713,7 @@
         <x:v>Polish / Indian-city / optional assets</x:v>
       </x:c>
       <x:c r="F10" s="27" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Ready</x:v>
       </x:c>
       <x:c r="G10" s="26"/>
     </x:row>
@@ -2734,7 +2734,7 @@
         <x:v>Polish / Indian-city / optional assets</x:v>
       </x:c>
       <x:c r="F11" s="27" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Ready</x:v>
       </x:c>
       <x:c r="G11" s="26"/>
     </x:row>
@@ -2755,7 +2755,7 @@
         <x:v>Polish / Indian-city / optional assets</x:v>
       </x:c>
       <x:c r="F12" s="27" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Ready</x:v>
       </x:c>
       <x:c r="G12" s="26"/>
     </x:row>
@@ -2776,7 +2776,7 @@
         <x:v>Polish / Indian-city / optional assets</x:v>
       </x:c>
       <x:c r="F13" s="27" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Ready</x:v>
       </x:c>
       <x:c r="G13" s="26"/>
     </x:row>

</xml_diff>